<commit_message>
Prepare Excel workbook for immediate use with error checks
Update Excel workbook metadata, clear example data from sheets (clients, vehicles, drivers, orders, dispatches, production, receipts, fuel), and set opening stock for materials to zero.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: 9e2e1c79-23df-4d0c-8254-b10e9f962356
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 9f01cd94-a924-4f40-b873-a1830365d861
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/a96ea08d-ecc7-4cdd-a8a2-07e393136f9a/9e2e1c79-23df-4d0c-8254-b10e9f962356/IYQPyUX
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/excel-deliverable/RMC-Plant-Daily-Workbook.xlsx
+++ b/excel-deliverable/RMC-Plant-Daily-Workbook.xlsx
@@ -1118,29 +1118,11 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>B-101</t>
-        </is>
-      </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>M25</t>
-        </is>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" s="21" t="inlineStr">
-        <is>
-          <t>Anil</t>
-        </is>
-      </c>
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="21" t="n"/>
       <c r="F5" s="23">
         <f>IFERROR(IF(OR(C5="",D5=""),"",D5*VLOOKUP(C5,'Setup - Mix Design'!$A$5:$I$304,2,0)),"")</f>
         <v/>
@@ -1167,29 +1149,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>B-102</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>M25</t>
-        </is>
-      </c>
-      <c r="D6" s="22" t="n">
-        <v>7</v>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>Anil</t>
-        </is>
-      </c>
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="21" t="n"/>
       <c r="F6" s="23">
         <f>IFERROR(IF(OR(C6="",D6=""),"",D6*VLOOKUP(C6,'Setup - Mix Design'!$A$5:$I$304,2,0)),"")</f>
         <v/>
@@ -1216,29 +1180,11 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>B-103</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>M30</t>
-        </is>
-      </c>
-      <c r="D7" s="22" t="n">
-        <v>7</v>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>Prakash</t>
-        </is>
-      </c>
+      <c r="A7" s="26" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="22" t="n"/>
+      <c r="E7" s="21" t="n"/>
       <c r="F7" s="23">
         <f>IFERROR(IF(OR(C7="",D7=""),"",D7*VLOOKUP(C7,'Setup - Mix Design'!$A$5:$I$304,2,0)),"")</f>
         <v/>
@@ -10576,112 +10522,52 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>Cement</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="n">
-        <v>30000</v>
-      </c>
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="22" t="n"/>
       <c r="D5" s="23">
         <f>IFERROR(IF(B5="","",VLOOKUP(B5,'Setup - Materials'!$A$5:$D$304,2,0)),"")</f>
         <v/>
       </c>
-      <c r="E5" s="22" t="n">
-        <v>7.4</v>
-      </c>
+      <c r="E5" s="22" t="n"/>
       <c r="F5" s="23">
         <f>IF(OR(C5="",E5=""),"",C5*E5)</f>
         <v/>
       </c>
-      <c r="G5" s="21" t="inlineStr">
-        <is>
-          <t>UltraTech</t>
-        </is>
-      </c>
-      <c r="H5" s="21" t="inlineStr">
-        <is>
-          <t>INV-5567</t>
-        </is>
-      </c>
+      <c r="G5" s="21" t="n"/>
+      <c r="H5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-21</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>Sand</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="n">
-        <v>60000</v>
-      </c>
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="22" t="n"/>
       <c r="D6" s="23">
         <f>IFERROR(IF(B6="","",VLOOKUP(B6,'Setup - Materials'!$A$5:$D$304,2,0)),"")</f>
         <v/>
       </c>
-      <c r="E6" s="22" t="n">
-        <v>1.15</v>
-      </c>
+      <c r="E6" s="22" t="n"/>
       <c r="F6" s="23">
         <f>IF(OR(C6="",E6=""),"",C6*E6)</f>
         <v/>
       </c>
-      <c r="G6" s="21" t="inlineStr">
-        <is>
-          <t>Krishna Sand</t>
-        </is>
-      </c>
-      <c r="H6" s="21" t="inlineStr">
-        <is>
-          <t>INV-2231</t>
-        </is>
-      </c>
+      <c r="G6" s="21" t="n"/>
+      <c r="H6" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-20</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Diesel</t>
-        </is>
-      </c>
-      <c r="C7" s="22" t="n">
-        <v>1000</v>
-      </c>
+      <c r="A7" s="26" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="22" t="n"/>
       <c r="D7" s="23">
         <f>IFERROR(IF(B7="","",VLOOKUP(B7,'Setup - Materials'!$A$5:$D$304,2,0)),"")</f>
         <v/>
       </c>
-      <c r="E7" s="22" t="n">
-        <v>92</v>
-      </c>
+      <c r="E7" s="22" t="n"/>
       <c r="F7" s="23">
         <f>IF(OR(C7="",E7=""),"",C7*E7)</f>
         <v/>
       </c>
-      <c r="G7" s="21" t="inlineStr">
-        <is>
-          <t>HP Petrol Pump</t>
-        </is>
-      </c>
-      <c r="H7" s="21" t="inlineStr">
-        <is>
-          <t>INV-9981</t>
-        </is>
-      </c>
+      <c r="G7" s="21" t="n"/>
+      <c r="H7" s="21" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="26" t="n"/>
@@ -15532,64 +15418,28 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>MH12 AB 1234</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="n">
-        <v>40</v>
-      </c>
-      <c r="D5" s="22" t="n">
-        <v>84120</v>
-      </c>
-      <c r="E5" s="22" t="n">
-        <v>92</v>
-      </c>
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="22" t="n"/>
+      <c r="E5" s="22" t="n"/>
       <c r="F5" s="23">
         <f>IF(OR(C5="",E5=""),"",C5*E5)</f>
         <v/>
       </c>
-      <c r="G5" s="21" t="inlineStr">
-        <is>
-          <t>Anil</t>
-        </is>
-      </c>
+      <c r="G5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>MH12 CD 5678</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="n">
-        <v>45</v>
-      </c>
-      <c r="D6" s="22" t="n">
-        <v>91250</v>
-      </c>
-      <c r="E6" s="22" t="n">
-        <v>92</v>
-      </c>
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="22" t="n"/>
+      <c r="E6" s="22" t="n"/>
       <c r="F6" s="23">
         <f>IF(OR(C6="",E6=""),"",C6*E6)</f>
         <v/>
       </c>
-      <c r="G6" s="21" t="inlineStr">
-        <is>
-          <t>Anil</t>
-        </is>
-      </c>
+      <c r="G6" s="21" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="26" t="n"/>
@@ -19929,85 +19779,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
-        <is>
-          <t>Skyline Builders Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>R. Mehta</t>
-        </is>
-      </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>9876543210</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr">
-        <is>
-          <t>27AABCS1234A1Z5</t>
-        </is>
-      </c>
-      <c r="E5" s="21" t="inlineStr">
-        <is>
-          <t>Plot 14, MIDC, Pune</t>
-        </is>
-      </c>
+      <c r="A5" s="21" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
-        <is>
-          <t>Greenfield Infra</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>S. Kulkarni</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>9822011223</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>27AAFCG5678B1Z2</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>Hinjewadi Phase 2, Pune</t>
-        </is>
-      </c>
+      <c r="A6" s="21" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>Metro Constructions</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>A. Shaikh</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>9890098900</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>27AADCM4321C1Z9</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>Wakad, Pune</t>
-        </is>
-      </c>
+      <c r="A7" s="21" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="21" t="n"/>
@@ -26579,79 +26369,25 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
-        <is>
-          <t>MH12 AB 1234</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>Transit Mixer</t>
-        </is>
-      </c>
-      <c r="C5" s="22" t="n">
-        <v>6</v>
-      </c>
-      <c r="D5" s="21" t="inlineStr">
-        <is>
-          <t>Ramesh Pawar</t>
-        </is>
-      </c>
-      <c r="E5" s="21" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
+      <c r="A5" s="21" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="22" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
-        <is>
-          <t>MH12 CD 5678</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>Transit Mixer</t>
-        </is>
-      </c>
-      <c r="C6" s="22" t="n">
-        <v>7</v>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>Suresh Jadhav</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
+      <c r="A6" s="21" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="22" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>MH12 EF 9012</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>Concrete Pump</t>
-        </is>
-      </c>
-      <c r="C7" s="22" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>Vijay More</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>Active</t>
-        </is>
-      </c>
+      <c r="A7" s="21" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="22" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="21" t="n"/>
@@ -28805,58 +28541,22 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="21" t="inlineStr">
-        <is>
-          <t>Ramesh Pawar</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>9001122334</t>
-        </is>
-      </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>MH1220190001234</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr"/>
+      <c r="A5" s="21" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="21" t="inlineStr">
-        <is>
-          <t>Suresh Jadhav</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>9002233445</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>MH1220180005678</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr"/>
+      <c r="A6" s="21" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>Vijay More</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>9003344556</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>MH1220200009012</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr"/>
+      <c r="A7" s="21" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="21" t="n"/>
@@ -30719,7 +30419,7 @@
         </is>
       </c>
       <c r="C5" s="22" t="n">
-        <v>50000</v>
+        <v>0</v>
       </c>
       <c r="D5" s="24" t="n">
         <v>7.5</v>
@@ -30737,7 +30437,7 @@
         </is>
       </c>
       <c r="C6" s="22" t="n">
-        <v>120000</v>
+        <v>0</v>
       </c>
       <c r="D6" s="24" t="n">
         <v>1.2</v>
@@ -30755,7 +30455,7 @@
         </is>
       </c>
       <c r="C7" s="22" t="n">
-        <v>150000</v>
+        <v>0</v>
       </c>
       <c r="D7" s="24" t="n">
         <v>1</v>
@@ -30773,7 +30473,7 @@
         </is>
       </c>
       <c r="C8" s="22" t="n">
-        <v>90000</v>
+        <v>0</v>
       </c>
       <c r="D8" s="24" t="n">
         <v>1.1</v>
@@ -30791,7 +30491,7 @@
         </is>
       </c>
       <c r="C9" s="22" t="n">
-        <v>800</v>
+        <v>0</v>
       </c>
       <c r="D9" s="24" t="n">
         <v>95</v>
@@ -30809,7 +30509,7 @@
         </is>
       </c>
       <c r="C10" s="22" t="n">
-        <v>2000</v>
+        <v>0</v>
       </c>
       <c r="D10" s="24" t="n">
         <v>92</v>
@@ -32703,34 +32403,12 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>ORD-0001</t>
-        </is>
-      </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>Skyline Builders Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr">
-        <is>
-          <t>Tower A, Kharadi</t>
-        </is>
-      </c>
-      <c r="E5" s="21" t="inlineStr">
-        <is>
-          <t>M25</t>
-        </is>
-      </c>
-      <c r="F5" s="22" t="n">
-        <v>30</v>
-      </c>
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="22" t="n"/>
       <c r="G5" s="23">
         <f>IFERROR(IF(E5="","",VLOOKUP(E5,'Setup - Mix Design'!$A$5:$I$304,9,0)),"")</f>
         <v/>
@@ -32753,34 +32431,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>ORD-0002</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>Greenfield Infra</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>Block C, Hinjewadi</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>M30</t>
-        </is>
-      </c>
-      <c r="F6" s="22" t="n">
-        <v>45</v>
-      </c>
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="22" t="n"/>
       <c r="G6" s="23">
         <f>IFERROR(IF(E6="","",VLOOKUP(E6,'Setup - Mix Design'!$A$5:$I$304,9,0)),"")</f>
         <v/>
@@ -32803,34 +32459,12 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-23</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>ORD-0003</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>Metro Constructions</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>Metro Pillar 212</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>M20</t>
-        </is>
-      </c>
-      <c r="F7" s="22" t="n">
-        <v>20</v>
-      </c>
+      <c r="A7" s="26" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="22" t="n"/>
       <c r="G7" s="23">
         <f>IFERROR(IF(E7="","",VLOOKUP(E7,'Setup - Mix Design'!$A$5:$I$304,9,0)),"")</f>
         <v/>
@@ -41300,39 +40934,13 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B5" s="21" t="inlineStr">
-        <is>
-          <t>CH-0001</t>
-        </is>
-      </c>
-      <c r="C5" s="21" t="inlineStr">
-        <is>
-          <t>ORD-0001</t>
-        </is>
-      </c>
-      <c r="D5" s="21" t="inlineStr">
-        <is>
-          <t>Skyline Builders Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="E5" s="21" t="inlineStr">
-        <is>
-          <t>M25</t>
-        </is>
-      </c>
-      <c r="F5" s="22" t="n">
-        <v>6</v>
-      </c>
-      <c r="G5" s="21" t="inlineStr">
-        <is>
-          <t>MH12 AB 1234</t>
-        </is>
-      </c>
+      <c r="A5" s="26" t="n"/>
+      <c r="B5" s="21" t="n"/>
+      <c r="C5" s="21" t="n"/>
+      <c r="D5" s="21" t="n"/>
+      <c r="E5" s="21" t="n"/>
+      <c r="F5" s="22" t="n"/>
+      <c r="G5" s="21" t="n"/>
       <c r="H5" s="23">
         <f>IFERROR(IF(G5="","",VLOOKUP(G5,'Setup - Vehicles'!$A$5:$D$304,4,0)),"")</f>
         <v/>
@@ -41345,46 +40953,16 @@
         <f>IF(OR(F5="",I5=""),"",F5*I5)</f>
         <v/>
       </c>
-      <c r="K5" s="21" t="inlineStr">
-        <is>
-          <t>Delivered</t>
-        </is>
-      </c>
+      <c r="K5" s="21" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B6" s="21" t="inlineStr">
-        <is>
-          <t>CH-0002</t>
-        </is>
-      </c>
-      <c r="C6" s="21" t="inlineStr">
-        <is>
-          <t>ORD-0001</t>
-        </is>
-      </c>
-      <c r="D6" s="21" t="inlineStr">
-        <is>
-          <t>Skyline Builders Pvt Ltd</t>
-        </is>
-      </c>
-      <c r="E6" s="21" t="inlineStr">
-        <is>
-          <t>M25</t>
-        </is>
-      </c>
-      <c r="F6" s="22" t="n">
-        <v>7</v>
-      </c>
-      <c r="G6" s="21" t="inlineStr">
-        <is>
-          <t>MH12 CD 5678</t>
-        </is>
-      </c>
+      <c r="A6" s="26" t="n"/>
+      <c r="B6" s="21" t="n"/>
+      <c r="C6" s="21" t="n"/>
+      <c r="D6" s="21" t="n"/>
+      <c r="E6" s="21" t="n"/>
+      <c r="F6" s="22" t="n"/>
+      <c r="G6" s="21" t="n"/>
       <c r="H6" s="23">
         <f>IFERROR(IF(G6="","",VLOOKUP(G6,'Setup - Vehicles'!$A$5:$D$304,4,0)),"")</f>
         <v/>
@@ -41397,46 +40975,16 @@
         <f>IF(OR(F6="",I6=""),"",F6*I6)</f>
         <v/>
       </c>
-      <c r="K6" s="21" t="inlineStr">
-        <is>
-          <t>Delivered</t>
-        </is>
-      </c>
+      <c r="K6" s="21" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="26" t="inlineStr">
-        <is>
-          <t>2026-06-22</t>
-        </is>
-      </c>
-      <c r="B7" s="21" t="inlineStr">
-        <is>
-          <t>CH-0003</t>
-        </is>
-      </c>
-      <c r="C7" s="21" t="inlineStr">
-        <is>
-          <t>ORD-0002</t>
-        </is>
-      </c>
-      <c r="D7" s="21" t="inlineStr">
-        <is>
-          <t>Greenfield Infra</t>
-        </is>
-      </c>
-      <c r="E7" s="21" t="inlineStr">
-        <is>
-          <t>M30</t>
-        </is>
-      </c>
-      <c r="F7" s="22" t="n">
-        <v>7</v>
-      </c>
-      <c r="G7" s="21" t="inlineStr">
-        <is>
-          <t>MH12 CD 5678</t>
-        </is>
-      </c>
+      <c r="A7" s="26" t="n"/>
+      <c r="B7" s="21" t="n"/>
+      <c r="C7" s="21" t="n"/>
+      <c r="D7" s="21" t="n"/>
+      <c r="E7" s="21" t="n"/>
+      <c r="F7" s="22" t="n"/>
+      <c r="G7" s="21" t="n"/>
       <c r="H7" s="23">
         <f>IFERROR(IF(G7="","",VLOOKUP(G7,'Setup - Vehicles'!$A$5:$D$304,4,0)),"")</f>
         <v/>
@@ -41449,11 +40997,7 @@
         <f>IF(OR(F7="",I7=""),"",F7*I7)</f>
         <v/>
       </c>
-      <c r="K7" s="21" t="inlineStr">
-        <is>
-          <t>Dispatched</t>
-        </is>
-      </c>
+      <c r="K7" s="21" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="26" t="n"/>

</xml_diff>